<commit_message>
verification IF + IF/ID is done
</commit_message>
<xml_diff>
--- a/RVI20U32/Docs/Plantilla_Verificacion_RV32I_5Etapas_IF_BRAM.xlsx
+++ b/RVI20U32/Docs/Plantilla_Verificacion_RV32I_5Etapas_IF_BRAM.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
-    <sheet name="Inicio_Guia" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Documentos_Entradas" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Matriz_RV32I" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Escenarios_Prueba" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Cobertura_Modulos" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Dashboard" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="MMIO_Interrupts_Traps" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Listas" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="Pipeline_5Etapas" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="Hazards_Forwarding" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="Inicio_Guia" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Documentos_Entradas" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Matriz_RV32I" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Escenarios_Prueba" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="Cobertura_Modulos" sheetId="5" state="visible" r:id="rId6"/>
+    <sheet name="Dashboard" sheetId="6" state="visible" r:id="rId7"/>
+    <sheet name="MMIO_Interrupts_Traps" sheetId="7" state="visible" r:id="rId8"/>
+    <sheet name="Listas" sheetId="8" state="visible" r:id="rId9"/>
+    <sheet name="Pipeline_5Etapas" sheetId="9" state="visible" r:id="rId10"/>
+    <sheet name="Hazards_Forwarding" sheetId="10" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1192" uniqueCount="600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1195" uniqueCount="602">
   <si>
     <t xml:space="preserve">Plantilla de verificación RV32I para core pipeline de 5 etapas con IF de 2 ciclos (BRAM síncrona)</t>
   </si>
@@ -1138,6 +1138,31 @@
     jal x0, done</t>
   </si>
   <si>
+    <t xml:space="preserve">.section .text.start
+.globl _start
+_start:
+    addi x1, x0, 5
+    addi x2, x0, 5
+    beq  x1, x2, target
+    addi x10, x0, 0x0A
+    addi x11, x0, 0x0B
+    addi x12, x0, 0x0C
+    addi x13, x0, 0x0D
+    addi x14, x0, 0x0E
+target:
+    addi x20, x0, 0x1A
+    addi x21, x0, 0x1B
+    addi x22, x0, 0x1C
+    addi x23, x0, 0x1D
+    addi x24, x0, 0x1E
+done:
+    jal x0, done
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WB → OK</t>
+  </si>
+  <si>
     <t xml:space="preserve">Descripción</t>
   </si>
   <si>
@@ -1156,6 +1181,9 @@
     <t xml:space="preserve">Fetch, PC, reset vector, redirect</t>
   </si>
   <si>
+    <t xml:space="preserve">Completado</t>
+  </si>
+  <si>
     <t xml:space="preserve">Registro de pipeline y flush/hold</t>
   </si>
   <si>
@@ -1274,9 +1302,6 @@
   </si>
   <si>
     <t xml:space="preserve">Bloqueado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Completado</t>
   </si>
   <si>
     <t xml:space="preserve">Docs</t>
@@ -2011,7 +2036,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2072,21 +2097,25 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Excel Built-in Explanatory Text" xfId="20"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3" customBuiltin="false"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6" customBuiltin="false"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4" customBuiltin="false"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7" customBuiltin="false"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5" customBuiltin="false"/>
+    <cellStyle name="Excel Built-in Explanatory Text" xfId="20" builtinId="53" customBuiltin="true"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="2">
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -2120,36 +2149,6 @@
         <charset val="1"/>
         <family val="2"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Lohit Devanagari"/>
-        <charset val="1"/>
-        <family val="2"/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F4E78"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <colors>
@@ -2215,7 +2214,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -2227,17 +2226,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
-                <a:uFillTx/>
-                <a:latin typeface="Arial"/>
+              <a:defRPr b="1" lang="es-ES" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="es-ES" sz="1800" b="1" u="none" strike="noStrike">
+              <a:rPr b="1" lang="es-ES" sz="1800" spc="-1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
                 <a:ea typeface="Calibri"/>
               </a:rPr>
@@ -2249,7 +2250,7 @@
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
-        <a:ln w="0">
+        <a:ln>
           <a:noFill/>
         </a:ln>
       </c:spPr>
@@ -2284,31 +2285,14 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
-            <c:txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
-                    <a:uFillTx/>
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-              </a:p>
-            </c:txPr>
+            <c:numFmt formatCode="General" sourceLinked="1"/>
             <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator>; </c:separator>
             <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="0"/>
-              </c:ext>
-            </c:extLst>
           </c:dLbls>
           <c:cat>
             <c:strRef>
@@ -2360,11 +2344,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="52399148"/>
-        <c:axId val="64857148"/>
+        <c:axId val="8450327"/>
+        <c:axId val="57998876"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="52399148"/>
+        <c:axId val="8450327"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2380,7 +2364,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2397,26 +2381,24 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr lang="es-ES" sz="1000" b="0" u="none" strike="noStrike">
+              <a:defRPr b="0" lang="es-ES" sz="1000" spc="-1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
                 <a:ea typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64857148"/>
+        <c:crossAx val="57998876"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="64857148"/>
+        <c:axId val="57998876"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2449,26 +2431,24 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr lang="es-ES" sz="1000" b="0" u="none" strike="noStrike">
+              <a:defRPr b="0" lang="es-ES" sz="1000" spc="-1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
                 <a:ea typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52399148"/>
+        <c:crossAx val="8450327"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
         <a:solidFill>
           <a:srgbClr val="ffffff"/>
         </a:solidFill>
-        <a:ln w="0">
+        <a:ln>
           <a:noFill/>
         </a:ln>
       </c:spPr>
@@ -2478,7 +2458,7 @@
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
-        <a:ln w="0">
+        <a:ln>
           <a:noFill/>
         </a:ln>
       </c:spPr>
@@ -2487,11 +2467,10 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr lang="es-ES" sz="1000" b="0" u="none" strike="noStrike">
+            <a:defRPr b="0" lang="es-ES" sz="1000" spc="-1" strike="noStrike">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:uFillTx/>
               <a:latin typeface="Calibri"/>
               <a:ea typeface="Calibri"/>
             </a:defRPr>
@@ -2516,7 +2495,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -2528,17 +2507,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
-                <a:uFillTx/>
-                <a:latin typeface="Arial"/>
+              <a:defRPr b="1" lang="es-ES" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="es-ES" sz="1800" b="1" u="none" strike="noStrike">
+              <a:rPr b="1" lang="es-ES" sz="1800" spc="-1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
                 <a:ea typeface="Calibri"/>
               </a:rPr>
@@ -2550,7 +2531,7 @@
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
-        <a:ln w="0">
+        <a:ln>
           <a:noFill/>
         </a:ln>
       </c:spPr>
@@ -2585,31 +2566,14 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
-            <c:txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
-                    <a:uFillTx/>
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-              </a:p>
-            </c:txPr>
+            <c:numFmt formatCode="0%" sourceLinked="1"/>
             <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator>; </c:separator>
             <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="0"/>
-              </c:ext>
-            </c:extLst>
           </c:dLbls>
           <c:cat>
             <c:strRef>
@@ -2662,13 +2626,13 @@
             <c:numRef>
               <c:f>Dashboard!$E$11:$E$23</c:f>
               <c:numCache>
-                <c:formatCode>0%</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2709,11 +2673,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="83459522"/>
-        <c:axId val="58780389"/>
+        <c:axId val="84834643"/>
+        <c:axId val="60193167"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="83459522"/>
+        <c:axId val="84834643"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2729,7 +2693,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2746,26 +2710,24 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr lang="es-ES" sz="1000" b="0" u="none" strike="noStrike">
+              <a:defRPr b="0" lang="es-ES" sz="1000" spc="-1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
                 <a:ea typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58780389"/>
+        <c:crossAx val="60193167"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58780389"/>
+        <c:axId val="60193167"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2798,26 +2760,24 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr lang="es-ES" sz="1000" b="0" u="none" strike="noStrike">
+              <a:defRPr b="0" lang="es-ES" sz="1000" spc="-1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
                 <a:ea typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83459522"/>
+        <c:crossAx val="84834643"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
         <a:solidFill>
           <a:srgbClr val="ffffff"/>
         </a:solidFill>
-        <a:ln w="0">
+        <a:ln>
           <a:noFill/>
         </a:ln>
       </c:spPr>
@@ -2827,7 +2787,7 @@
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
-        <a:ln w="0">
+        <a:ln>
           <a:noFill/>
         </a:ln>
       </c:spPr>
@@ -2836,11 +2796,10 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr lang="es-ES" sz="1000" b="0" u="none" strike="noStrike">
+            <a:defRPr b="0" lang="es-ES" sz="1000" spc="-1" strike="noStrike">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:uFillTx/>
               <a:latin typeface="Calibri"/>
               <a:ea typeface="Calibri"/>
             </a:defRPr>
@@ -2876,13 +2835,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>6754320</xdr:colOff>
+      <xdr:colOff>6753600</xdr:colOff>
       <xdr:row>48</xdr:row>
-      <xdr:rowOff>72000</xdr:rowOff>
+      <xdr:rowOff>71280</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Imagen 1"/>
+        <xdr:cNvPr id="0" name="Imagen 1" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2891,14 +2850,13 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1969200" y="9150480"/>
-          <a:ext cx="18111960" cy="3266640"/>
+          <a:off x="1969560" y="9150480"/>
+          <a:ext cx="18123840" cy="3265560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:ln>
           <a:noFill/>
         </a:ln>
       </xdr:spPr>
@@ -2914,13 +2872,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>7017480</xdr:colOff>
+      <xdr:colOff>7016760</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>156240</xdr:rowOff>
+      <xdr:rowOff>155520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 2"/>
+        <xdr:cNvPr id="1" name="Imagen 2" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2929,14 +2887,13 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2056680" y="5150160"/>
-          <a:ext cx="18287640" cy="3366360"/>
+          <a:off x="2058120" y="5149800"/>
+          <a:ext cx="18298440" cy="3366000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:ln>
           <a:noFill/>
         </a:ln>
       </xdr:spPr>
@@ -2952,13 +2909,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>6950880</xdr:colOff>
+      <xdr:colOff>6950160</xdr:colOff>
       <xdr:row>59</xdr:row>
-      <xdr:rowOff>176760</xdr:rowOff>
+      <xdr:rowOff>176040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 3"/>
+        <xdr:cNvPr id="2" name="Imagen 3" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2967,36 +2924,35 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2019240" y="13147920"/>
-          <a:ext cx="18258480" cy="3003480"/>
+          <a:off x="2020680" y="13147920"/>
+          <a:ext cx="18269280" cy="3002760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:ln>
           <a:noFill/>
         </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>23400</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>24120</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1321200</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>114840</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>6687360</xdr:colOff>
-      <xdr:row>70</xdr:row>
-      <xdr:rowOff>159480</xdr:rowOff>
+      <xdr:colOff>6945480</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>29520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 1"/>
+        <xdr:cNvPr id="3" name="Imagen 4" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3005,14 +2961,50 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2028240" y="16570440"/>
-          <a:ext cx="17985960" cy="3051000"/>
+          <a:off x="1981440" y="16470360"/>
+          <a:ext cx="18303840" cy="3686040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>6892200</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>58320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 5" descr=""/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2006280" y="20805120"/>
+          <a:ext cx="18225720" cy="4129920"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
           <a:noFill/>
         </a:ln>
       </xdr:spPr>
@@ -3033,9 +3025,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>757800</xdr:colOff>
+      <xdr:colOff>757080</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>131760</xdr:rowOff>
+      <xdr:rowOff>131040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3043,8 +3035,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="9521280" y="380880"/>
-        <a:ext cx="4906800" cy="3047760"/>
+        <a:off x="9531000" y="380880"/>
+        <a:ext cx="4913280" cy="3047040"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3063,9 +3055,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>757800</xdr:colOff>
+      <xdr:colOff>757080</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>6840</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3073,8 +3065,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="9521280" y="3619440"/>
-        <a:ext cx="4906800" cy="3999960"/>
+        <a:off x="9531000" y="3619080"/>
+        <a:ext cx="4913280" cy="3999240"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3105,119 +3097,13 @@
 </table>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
-  <a:themeElements>
-    <a:clrScheme name="LibreOffice">
-      <a:dk1>
-        <a:srgbClr val="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:srgbClr val="ffffff"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="000000"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="ffffff"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="18a303"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="0369a3"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="a33e03"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8e03a3"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="c99c00"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="c9211e"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000ee"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="551a8b"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme>
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L13"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="129.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="178.59"/>
@@ -3463,8 +3349,8 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3473,12 +3359,12 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L9"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.33"/>
@@ -3495,7 +3381,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>226</v>
@@ -3504,22 +3390,22 @@
         <v>222</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>225</v>
@@ -3533,34 +3419,34 @@
     </row>
     <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>310</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>237</v>
@@ -3571,34 +3457,34 @@
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>310</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>104</v>
@@ -3609,34 +3495,34 @@
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>316</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>237</v>
@@ -3647,34 +3533,34 @@
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>253</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>237</v>
@@ -3685,34 +3571,34 @@
     </row>
     <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>104</v>
@@ -3723,34 +3609,34 @@
     </row>
     <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>104</v>
@@ -3761,22 +3647,22 @@
     </row>
     <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>230</v>
@@ -3785,10 +3671,10 @@
         <v>253</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>237</v>
@@ -3799,34 +3685,34 @@
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>166</v>
@@ -3837,8 +3723,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3847,12 +3733,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L13"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="64.09"/>
@@ -4257,14 +4143,14 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F11" type="list">
+    <dataValidation allowBlank="false" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F11" type="list">
       <formula1>Listas!$A$2:$A$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -4273,12 +4159,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N41"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.64"/>
@@ -5974,26 +5860,26 @@
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>K2="Bloqueado"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>K2="No iniciado"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>K2="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K41" type="list">
+    <dataValidation allowBlank="false" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K41" type="list">
       <formula1>Listas!$A$2:$A$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M2:M41" type="list">
+    <dataValidation allowBlank="false" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M2:M41" type="list">
       <formula1>Listas!$B$2:$B$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -6002,18 +5888,18 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:M87"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="72.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="36.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="72.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="36.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="33.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="101.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13.33"/>
@@ -6815,6 +6701,63 @@
         <v>357</v>
       </c>
     </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B64" s="14"/>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B65" s="14"/>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B66" s="14"/>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B67" s="14"/>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B68" s="14"/>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B69" s="14"/>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B70" s="14"/>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B71" s="14"/>
+    </row>
+    <row r="72" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B72" s="14"/>
+    </row>
+    <row r="73" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B73" s="14"/>
+    </row>
+    <row r="74" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B74" s="14"/>
+    </row>
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B75" s="14"/>
+    </row>
+    <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B76" s="14"/>
+    </row>
+    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B77" s="14"/>
+    </row>
+    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="15" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="260.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="14" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C87" s="13" t="s">
+        <v>359</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="J2:J21">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -6823,37 +6766,37 @@
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>J2="En progreso"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>J2="Bloqueado"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>J2="No iniciado"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>J2="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H2:H20" type="list">
+    <dataValidation allowBlank="false" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H2:H20" type="list">
       <formula1>Listas!$C$2:$C$8</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I2:I20" type="list">
+    <dataValidation allowBlank="false" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I2:I20" type="list">
       <formula1>Listas!$D$2:$D$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J2:J20" type="list">
+    <dataValidation allowBlank="false" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J2:J20" type="list">
       <formula1>Listas!$A$2:$A$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K20" type="list">
+    <dataValidation allowBlank="false" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K20" type="list">
       <formula1>Listas!$B$2:$B$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -6863,12 +6806,12 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="56.13"/>
@@ -6885,67 +6828,67 @@
         <v>220</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>92</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>230</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>4</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="15" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="E2" s="16" t="n">
+        <v>1</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>102</v>
+        <v>366</v>
       </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>253</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="E3" s="16" t="n">
+        <v>1</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>102</v>
+        <v>366</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
@@ -6955,7 +6898,7 @@
         <v>265</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>2</v>
@@ -6963,7 +6906,7 @@
       <c r="D4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -6977,7 +6920,7 @@
         <v>272</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>1</v>
@@ -6985,7 +6928,7 @@
       <c r="D5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="3" t="s">
@@ -6999,7 +6942,7 @@
         <v>280</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>1</v>
@@ -7007,7 +6950,7 @@
       <c r="D6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="3" t="s">
@@ -7018,10 +6961,10 @@
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>1</v>
@@ -7029,7 +6972,7 @@
       <c r="D7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="3" t="s">
@@ -7040,10 +6983,10 @@
     </row>
     <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>3</v>
@@ -7051,7 +6994,7 @@
       <c r="D8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="3" t="s">
@@ -7062,10 +7005,10 @@
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>4</v>
@@ -7073,7 +7016,7 @@
       <c r="D9" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="3" t="s">
@@ -7084,10 +7027,10 @@
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>4</v>
@@ -7095,7 +7038,7 @@
       <c r="D10" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="3" t="s">
@@ -7106,10 +7049,10 @@
     </row>
     <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>1</v>
@@ -7117,7 +7060,7 @@
       <c r="D11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="3" t="s">
@@ -7128,10 +7071,10 @@
     </row>
     <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>3</v>
@@ -7139,7 +7082,7 @@
       <c r="D12" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="3" t="s">
@@ -7153,7 +7096,7 @@
         <v>334</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>2</v>
@@ -7161,7 +7104,7 @@
       <c r="D13" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="3" t="s">
@@ -7172,10 +7115,10 @@
     </row>
     <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>1</v>
@@ -7183,7 +7126,7 @@
       <c r="D14" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="15" t="n">
+      <c r="E14" s="16" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="3" t="s">
@@ -7194,10 +7137,10 @@
     </row>
     <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>2</v>
@@ -7216,10 +7159,10 @@
     </row>
     <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>0</v>
@@ -7231,17 +7174,17 @@
         <v>0</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>0</v>
@@ -7253,7 +7196,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
@@ -7263,7 +7206,7 @@
         <v>348</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>2</v>
@@ -7288,10 +7231,10 @@
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>F2="En progreso"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>F2="Bloqueado"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>F2="No iniciado"</formula>
     </cfRule>
     <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -7307,20 +7250,20 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{904C8EBB-B655-4444-83BD-584A58B0C0B5}</x14:id>
+          <x14:id>{D6DEC475-22AB-4C2F-B295-48816196CBC8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F14" type="list">
+    <dataValidation allowBlank="false" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F14" type="list">
       <formula1>Listas!$A$2:$A$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7329,7 +7272,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{904C8EBB-B655-4444-83BD-584A58B0C0B5}">
+          <x14:cfRule type="dataBar" id="{D6DEC475-22AB-4C2F-B295-48816196CBC8}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -7346,12 +7289,12 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N23"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.17"/>
@@ -7365,28 +7308,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
@@ -7413,10 +7356,10 @@
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -7433,7 +7376,7 @@
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B4" s="3" t="n">
         <f aca="false">COUNTA(Matriz_RV32I!B2:B100)</f>
@@ -7454,7 +7397,7 @@
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B5" s="3" t="n">
         <f aca="false">COUNTIF(Matriz_RV32I!K2:K100,"Completado")</f>
@@ -7475,9 +7418,9 @@
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="B6" s="15" t="n">
+        <v>399</v>
+      </c>
+      <c r="B6" s="16" t="n">
         <f aca="false">IFERROR(B5/B4,0)</f>
         <v>0</v>
       </c>
@@ -7496,11 +7439,11 @@
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="B7" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="B7" s="16" t="n">
         <f aca="false">IFERROR(COUNTIF(Cobertura_Modulos!F2:F100,"Completado")/COUNTIF(Cobertura_Modulos!F2:F100,"&lt;&gt;N/A"),0)</f>
-        <v>0</v>
+        <v>0.0206185567010309</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
@@ -7517,7 +7460,7 @@
     </row>
     <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="B8" s="3" t="n">
         <f aca="false">COUNTIF(Hazards_Forwarding!L2:L100,"Completado")</f>
@@ -7538,10 +7481,10 @@
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B9" s="3" t="n">
-        <f aca="false">COUNTIF(Escenarios_Prueba!J2:J106,"Completado")</f>
+        <f aca="false">COUNTIF(Escenarios_Prueba!J2:J120,"Completado")</f>
         <v>0</v>
       </c>
       <c r="C9" s="3"/>
@@ -7562,17 +7505,17 @@
         <v>92</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="4" t="s">
         <v>220</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
@@ -7595,13 +7538,13 @@
       <c r="D11" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D11,Cobertura_Modulos!A:A,0)),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="3" t="str">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!D:D,MATCH(D11,Cobertura_Modulos!A:A,0)),0)&amp;"/"&amp;IFERROR(INDEX(Cobertura_Modulos!C:C,MATCH(D11,Cobertura_Modulos!A:A,0)),0)</f>
-        <v>0/4</v>
+        <v>4/4</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
@@ -7614,7 +7557,7 @@
     </row>
     <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B12" s="3" t="n">
         <f aca="false">COUNTIF(Matriz_RV32I!K2:K100,"En progreso")</f>
@@ -7624,13 +7567,13 @@
       <c r="D12" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D12,Cobertura_Modulos!A:A,0)),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" s="3" t="str">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!D:D,MATCH(D12,Cobertura_Modulos!A:A,0)),0)&amp;"/"&amp;IFERROR(INDEX(Cobertura_Modulos!C:C,MATCH(D12,Cobertura_Modulos!A:A,0)),0)</f>
-        <v>0/2</v>
+        <v>2/2</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
@@ -7643,7 +7586,7 @@
     </row>
     <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="B13" s="3" t="n">
         <f aca="false">COUNTIF(Matriz_RV32I!K2:K100,"Bloqueado")</f>
@@ -7653,7 +7596,7 @@
       <c r="D13" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D13,Cobertura_Modulos!A:A,0)),0)</f>
         <v>0</v>
       </c>
@@ -7672,7 +7615,7 @@
     </row>
     <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>404</v>
+        <v>366</v>
       </c>
       <c r="B14" s="3" t="n">
         <f aca="false">COUNTIF(Matriz_RV32I!K2:K100,"Completado")</f>
@@ -7682,7 +7625,7 @@
       <c r="D14" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="E14" s="15" t="n">
+      <c r="E14" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D14,Cobertura_Modulos!A:A,0)),0)</f>
         <v>0</v>
       </c>
@@ -7701,7 +7644,7 @@
     </row>
     <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B15" s="3" t="n">
         <f aca="false">COUNTIF(Matriz_RV32I!K2:K100,"N/A")</f>
@@ -7711,7 +7654,7 @@
       <c r="D15" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="E15" s="15" t="n">
+      <c r="E15" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D15,Cobertura_Modulos!A:A,0)),0)</f>
         <v>0</v>
       </c>
@@ -7730,16 +7673,16 @@
     </row>
     <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3" t="s">
-        <v>368</v>
-      </c>
-      <c r="E16" s="15" t="n">
+        <v>371</v>
+      </c>
+      <c r="E16" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D16,Cobertura_Modulos!A:A,0)),0)</f>
         <v>0</v>
       </c>
@@ -7758,7 +7701,7 @@
     </row>
     <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B17" s="3" t="n">
         <f aca="false">COUNTIF(Documentos_Entradas!D2:D100,"Sí")</f>
@@ -7766,9 +7709,9 @@
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3" t="s">
-        <v>370</v>
-      </c>
-      <c r="E17" s="15" t="n">
+        <v>373</v>
+      </c>
+      <c r="E17" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D17,Cobertura_Modulos!A:A,0)),0)</f>
         <v>0</v>
       </c>
@@ -7787,7 +7730,7 @@
     </row>
     <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B18" s="4" t="n">
         <f aca="false">COUNTIFS(Documentos_Entradas!D2:D100,"Sí",Documentos_Entradas!I2:I100,"Completo")</f>
@@ -7795,9 +7738,9 @@
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3" t="s">
-        <v>372</v>
-      </c>
-      <c r="E18" s="15" t="n">
+        <v>375</v>
+      </c>
+      <c r="E18" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D18,Cobertura_Modulos!A:A,0)),0)</f>
         <v>0</v>
       </c>
@@ -7816,7 +7759,7 @@
     </row>
     <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B19" s="3" t="n">
         <f aca="false">COUNTA(MMIO_Interrupts_Traps!A2:A100)</f>
@@ -7824,9 +7767,9 @@
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3" t="s">
-        <v>374</v>
-      </c>
-      <c r="E19" s="15" t="n">
+        <v>377</v>
+      </c>
+      <c r="E19" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D19,Cobertura_Modulos!A:A,0)),0)</f>
         <v>0</v>
       </c>
@@ -7845,7 +7788,7 @@
     </row>
     <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B20" s="3" t="n">
         <f aca="false">COUNTIF(MMIO_Interrupts_Traps!J2:J100,"Completado")</f>
@@ -7853,9 +7796,9 @@
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="E20" s="15" t="n">
+        <v>381</v>
+      </c>
+      <c r="E20" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D20,Cobertura_Modulos!A:A,0)),0)</f>
         <v>0</v>
       </c>
@@ -7874,9 +7817,9 @@
     </row>
     <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="B21" s="15" t="n">
+        <v>412</v>
+      </c>
+      <c r="B21" s="16" t="n">
         <f aca="false">IFERROR(B20/B19,0)</f>
         <v>0</v>
       </c>
@@ -7884,7 +7827,7 @@
       <c r="D21" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="E21" s="15" t="n">
+      <c r="E21" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D21,Cobertura_Modulos!A:A,0)),0)</f>
         <v>0</v>
       </c>
@@ -7906,9 +7849,9 @@
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="E22" s="15" t="n">
+        <v>386</v>
+      </c>
+      <c r="E22" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D22,Cobertura_Modulos!A:A,0)),0)</f>
         <v>0</v>
       </c>
@@ -7927,12 +7870,12 @@
     </row>
     <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3"/>
-      <c r="B23" s="15"/>
+      <c r="B23" s="16"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3" t="s">
         <v>348</v>
       </c>
-      <c r="E23" s="15" t="n">
+      <c r="E23" s="16" t="n">
         <f aca="false">IFERROR(INDEX(Cobertura_Modulos!E:E,MATCH(D23,Cobertura_Modulos!A:A,0)),0)</f>
         <v>0</v>
       </c>
@@ -7962,14 +7905,14 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6DC2ACFC-46D7-4A79-8892-582C30E3B6B1}</x14:id>
+          <x14:id>{9389F077-D978-4CA6-81D8-80E9BB5053D1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7979,7 +7922,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6DC2ACFC-46D7-4A79-8892-582C30E3B6B1}">
+          <x14:cfRule type="dataBar" id="{9389F077-D978-4CA6-81D8-80E9BB5053D1}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -7996,12 +7939,12 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.12"/>
@@ -8018,31 +7961,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>220</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>92</v>
@@ -8053,22 +7996,22 @@
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>60</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>4</v>
@@ -8076,7 +8019,7 @@
       <c r="H2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I2" s="15" t="n">
+      <c r="I2" s="16" t="n">
         <f aca="false">IF(G2=0,0,H2/G2)</f>
         <v>0</v>
       </c>
@@ -8087,22 +8030,22 @@
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>60</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>8</v>
@@ -8110,7 +8053,7 @@
       <c r="H3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="15" t="n">
+      <c r="I3" s="16" t="n">
         <f aca="false">IF(G3=0,0,H3/G3)</f>
         <v>0</v>
       </c>
@@ -8121,22 +8064,22 @@
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>60</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>4</v>
@@ -8144,7 +8087,7 @@
       <c r="H4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="15" t="n">
+      <c r="I4" s="16" t="n">
         <f aca="false">IF(G4=0,0,H4/G4)</f>
         <v>0</v>
       </c>
@@ -8155,22 +8098,22 @@
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>63</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>8</v>
@@ -8178,7 +8121,7 @@
       <c r="H5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="15" t="n">
+      <c r="I5" s="16" t="n">
         <f aca="false">IF(G5=0,0,H5/G5)</f>
         <v>0</v>
       </c>
@@ -8189,22 +8132,22 @@
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>63</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>6</v>
@@ -8212,7 +8155,7 @@
       <c r="H6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="15" t="n">
+      <c r="I6" s="16" t="n">
         <f aca="false">IF(G6=0,0,H6/G6)</f>
         <v>0</v>
       </c>
@@ -8223,22 +8166,22 @@
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>63</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>4</v>
@@ -8246,7 +8189,7 @@
       <c r="H7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="15" t="n">
+      <c r="I7" s="16" t="n">
         <f aca="false">IF(G7=0,0,H7/G7)</f>
         <v>0</v>
       </c>
@@ -8257,16 +8200,16 @@
     </row>
     <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>216</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>67</v>
@@ -8280,7 +8223,7 @@
       <c r="H8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="15" t="n">
+      <c r="I8" s="16" t="n">
         <f aca="false">IF(G8=0,0,H8/G8)</f>
         <v>0</v>
       </c>
@@ -8291,16 +8234,16 @@
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>216</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>67</v>
@@ -8314,7 +8257,7 @@
       <c r="H9" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I9" s="15" t="n">
+      <c r="I9" s="16" t="n">
         <f aca="false">IF(G9=0,0,H9/G9)</f>
         <v>0</v>
       </c>
@@ -8325,16 +8268,16 @@
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>216</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>67</v>
@@ -8348,7 +8291,7 @@
       <c r="H10" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="15" t="n">
+      <c r="I10" s="16" t="n">
         <f aca="false">IF(G10=0,0,H10/G10)</f>
         <v>0</v>
       </c>
@@ -8359,16 +8302,16 @@
     </row>
     <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>216</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>67</v>
@@ -8382,7 +8325,7 @@
       <c r="H11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="15" t="n">
+      <c r="I11" s="16" t="n">
         <f aca="false">IF(G11=0,0,H11/G11)</f>
         <v>0</v>
       </c>
@@ -8418,20 +8361,20 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BDFDABC0-B840-44F9-8AED-17A2D0AAC8E3}</x14:id>
+          <x14:id>{77D06EF9-6D13-4C6A-A66A-273C8870D886}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J2:J11" type="list">
+    <dataValidation allowBlank="false" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J2:J11" type="list">
       <formula1>Listas!$A$2:$A$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -8443,7 +8386,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BDFDABC0-B840-44F9-8AED-17A2D0AAC8E3}">
+          <x14:cfRule type="dataBar" id="{77D06EF9-6D13-4C6A-A66A-273C8870D886}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -8460,12 +8403,12 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="1" style="1" width="22.69"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="5" style="1" width="10.77"/>
@@ -8479,10 +8422,10 @@
         <v>94</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8501,13 +8444,13 @@
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>166</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>38</v>
@@ -8515,7 +8458,7 @@
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>212</v>
@@ -8524,12 +8467,12 @@
         <v>349</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>404</v>
+        <v>366</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>237</v>
@@ -8541,7 +8484,7 @@
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3" t="s">
@@ -8553,7 +8496,7 @@
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="D7" s="3"/>
     </row>
@@ -8567,8 +8510,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -8577,12 +8520,12 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42.86"/>
@@ -8590,36 +8533,36 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="42.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="108.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="62.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="110.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="110.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="43.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="15.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="9.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="69.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="30.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="69.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="30.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="13" style="1" width="10.77"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>348</v>
@@ -8628,7 +8571,7 @@
         <v>92</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>33</v>
@@ -8637,62 +8580,62 @@
     </row>
     <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>102</v>
       </c>
       <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="L2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>102</v>
@@ -8703,28 +8646,28 @@
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>102</v>
@@ -8735,25 +8678,25 @@
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>140</v>
@@ -8767,28 +8710,28 @@
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>102</v>
@@ -8802,25 +8745,25 @@
         <v>253</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>102</v>
@@ -8831,28 +8774,28 @@
     </row>
     <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="D8" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>504</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>505</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>507</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>502</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>102</v>
@@ -8863,28 +8806,28 @@
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="H9" s="3" t="s">
         <v>504</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>508</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>509</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>510</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>511</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>502</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>102</v>
@@ -8898,25 +8841,25 @@
         <v>334</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>102</v>
@@ -8930,25 +8873,25 @@
         <v>341</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>102</v>
@@ -8959,42 +8902,42 @@
     </row>
     <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="J12" s="3"/>
       <c r="K12" s="3" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="L12" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
verification TC-014 + Extra
</commit_message>
<xml_diff>
--- a/RVI20U32/Docs/Plantilla_Verificacion_RV32I_5Etapas_IF_BRAM.xlsx
+++ b/RVI20U32/Docs/Plantilla_Verificacion_RV32I_5Etapas_IF_BRAM.xlsx
@@ -2456,7 +2456,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart19.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -2586,11 +2586,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="93862686"/>
-        <c:axId val="89121999"/>
+        <c:axId val="20156672"/>
+        <c:axId val="77796890"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="93862686"/>
+        <c:axId val="20156672"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2633,14 +2633,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89121999"/>
+        <c:crossAx val="77796890"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="89121999"/>
+        <c:axId val="77796890"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2683,7 +2683,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93862686"/>
+        <c:crossAx val="20156672"/>
         <c:crosses val="autoZero"/>
       </c:valAx>
       <c:spPr>
@@ -2737,7 +2737,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart20.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -2915,11 +2915,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="90707008"/>
-        <c:axId val="89598582"/>
+        <c:axId val="92808703"/>
+        <c:axId val="55203752"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="90707008"/>
+        <c:axId val="92808703"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2962,14 +2962,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89598582"/>
+        <c:crossAx val="55203752"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="89598582"/>
+        <c:axId val="55203752"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3012,7 +3012,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90707008"/>
+        <c:crossAx val="92808703"/>
         <c:crosses val="autoZero"/>
       </c:valAx>
       <c:spPr>
@@ -8061,7 +8061,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D34B7274-F94E-4A76-BEA8-C031F8237B2A}</x14:id>
+          <x14:id>{3ABEB029-9772-4E6D-AEEC-5FBFE2973957}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8083,7 +8083,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D34B7274-F94E-4A76-BEA8-C031F8237B2A}">
+          <x14:cfRule type="dataBar" id="{3ABEB029-9772-4E6D-AEEC-5FBFE2973957}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -8716,7 +8716,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EBDD3CC4-CF50-4749-AAE0-A41E449E6AD5}</x14:id>
+          <x14:id>{B9CF78B3-4E70-49BA-8F6D-B4B6B091ACE8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8733,7 +8733,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EBDD3CC4-CF50-4749-AAE0-A41E449E6AD5}">
+          <x14:cfRule type="dataBar" id="{B9CF78B3-4E70-49BA-8F6D-B4B6B091ACE8}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -9172,7 +9172,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{89C38499-92D2-4959-9C19-A4C0FB90508A}</x14:id>
+          <x14:id>{D5915D34-A471-486B-88D6-11BA2740B2AC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9197,7 +9197,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{89C38499-92D2-4959-9C19-A4C0FB90508A}">
+          <x14:cfRule type="dataBar" id="{D5915D34-A471-486B-88D6-11BA2740B2AC}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>

</xml_diff>